<commit_message>
RPA: pelny skan (pierwszy przerwal Transfermarkt przy 7 krajach) - 42 zawodnikow, doszli Ime Okon (Hannover 96), Devin Titus i Tshegofatso Mabasa (MAS Fes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/zawodnicy_za.xlsx
+++ b/zawodnicy_za.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -708,389 +708,440 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mhleli</t>
+          <t>Tshegofatso</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mabuza</t>
+          <t>Mabasa</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[Luksemburg] FC Differdange 03</t>
+          <t>[Maroko] MAS Fès</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Siviwe</t>
+          <t>Mhleli</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Magidigidi</t>
+          <t>Mabuza</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>[Belgia] Beerschot VA</t>
+          <t>[Luksemburg] FC Differdange 03</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Olwethu</t>
+          <t>Siviwe</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Makhanya</t>
+          <t>Magidigidi</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[Szkocja] Glasgow Rangers</t>
+          <t>[Belgia] Beerschot VA</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Thapelo</t>
+          <t>Olwethu</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Maseko</t>
+          <t>Makhanya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[Dania] FC København</t>
+          <t>[Szkocja] Glasgow Rangers</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Siyanda</t>
+          <t>Thapelo</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mathenjwa</t>
+          <t>Maseko</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>[Gruzja] FC Spaeri Tbilisi</t>
+          <t>[Dania] FC København</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mihlali</t>
+          <t>Siyanda</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mayambela</t>
+          <t>Mathenjwa</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>[Cypr] Omonia Nicosia</t>
+          <t>[Gruzja] FC Spaeri Tbilisi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Mihlali</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mbewe</t>
+          <t>Mayambela</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>[Bośnia i Hercegowina] FK Romanija Pale</t>
+          <t>[Cypr] Omonia Nicosia</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mbekezeli</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mbokazi</t>
+          <t>Mbewe</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] Chicago Fire FC</t>
+          <t>[Bośnia i Hercegowina] FK Romanija Pale</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sipho</t>
+          <t>Mbekezeli</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mbule</t>
+          <t>Mbokazi</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>[Irak] Zakho SC</t>
+          <t>[Stany Zjednaczone] Chicago Fire FC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aden</t>
+          <t>Sipho</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>McCarthy</t>
+          <t>Mbule</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>[Azerbejdżan] Sabah FK</t>
+          <t>[Irak] Zakho SC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Relebohile</t>
+          <t>Aden</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Mofokeng</t>
+          <t>McCarthy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>[Belgia] Union Saint-Gilloise</t>
+          <t>[Azerbejdżan] Sabah FK</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Siyabonga</t>
+          <t>Relebohile</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ngezana</t>
+          <t>Mofokeng</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>[Rumunia] FCSB</t>
+          <t>[Belgia] Union Saint-Gilloise</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cafú</t>
+          <t>Siyabonga</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Phete</t>
+          <t>Ngezana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>[Islandia] Vestri Ísafjördur</t>
+          <t>[Rumunia] FCSB</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Waylon</t>
+          <t>Ime</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Renecke</t>
+          <t>Okon</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>[Szwecja] Hammarby IF</t>
+          <t>[Niemcy] Hannover 96</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Jaedin</t>
+          <t>Cafú</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Rhodes</t>
+          <t>Phete</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>[Austria] SV Ried</t>
+          <t>[Islandia] Vestri Ísafjördur</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kgaogelo</t>
+          <t>Waylon</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Sekgota</t>
+          <t>Renecke</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>[Egipt] Petrojet-Suez</t>
+          <t>[Szwecja] Hammarby IF</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Luther</t>
+          <t>Jaedin</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Singh</t>
+          <t>Rhodes</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>[Cypr] AEL Limassol</t>
+          <t>[Austria] SV Ried</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Yaya</t>
+          <t>Kgaogelo</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Sithole</t>
+          <t>Sekgota</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>[Portugalia] CD Tondela</t>
+          <t>[Egipt] Petrojet-Suez</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Darren</t>
+          <t>Luther</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Singh</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] Detroit City FC</t>
+          <t>[Cypr] AEL Limassol</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tylon</t>
+          <t>Yaya</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Sithole</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] New England Revolution</t>
+          <t>[Portugalia] CD Tondela</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Marko</t>
+          <t>Darren</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Veselinovic</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>[Islandia] Leiknir Reykjavík</t>
+          <t>[Stany Zjednaczone] Detroit City FC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jamie</t>
+          <t>Tylon</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Webber</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>[Stany Zjednaczone] FC Tulsa</t>
+          <t>[Stany Zjednaczone] New England Revolution</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>Devin</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Titus</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>[Maroko] MAS Fès</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Marko</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Veselinovic</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>[Islandia] Leiknir Reykjavík</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Jamie</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Webber</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>[Stany Zjednaczone] FC Tulsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>Vuthlarhi</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Wisdom Baloyi</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>[Armenia] Lernayin Artsakh Goris</t>
         </is>

</xml_diff>